<commit_message>
feat: refresh PowerCare UI and inventory classification
</commit_message>
<xml_diff>
--- a/public/templates/spare-parts-import-template.xlsx
+++ b/public/templates/spare-parts-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare_Parts_Import" sheetId="1" r:id="R68f5e41e5a8a4472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="2" r:id="Rcc1857b24d2544fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างรหัสอ้างอิง" sheetId="3" r:id="R6184c330203748f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spare_Parts_Import" sheetId="1" r:id="R310bda14a1824d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="2" r:id="Rdb7d850513834b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างรหัสอ้างอิง" sheetId="3" r:id="R441b0945633f4f63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -84,6 +84,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8F5F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0E75BC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -211,7 +216,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -345,6 +350,17 @@
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -560,6 +576,7 @@
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="27.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -601,6 +618,9 @@
       </x:c>
       <x:c r="M1" s="6" t="str">
         <x:v>สถานะใช้งาน (Active TRUE/FALSE)</x:v>
+      </x:c>
+      <x:c r="N1" s="69" t="str">
+        <x:v>รหัสกลุ่มอะไหล่/วัสดุ (Material Group Code)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">

</xml_diff>